<commit_message>
Add some herbicide info
</commit_message>
<xml_diff>
--- a/data/data-wrangling-intermediate/21_treatment-info/model29-treatment-info.xlsx
+++ b/data/data-wrangling-intermediate/21_treatment-info/model29-treatment-info.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eltnmsu-my.sharepoint.com/personal/lossanna_nmsu_edu/Documents/Documents/04_LDC-LTDL/LDC-LTDL_v04/data/data-wrangling-intermediate/21_treatment-info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="8_{E2B0E8AA-A2DA-4D30-8834-36D20A8CC477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B547BEF-056C-42C7-AA8C-1C97321F421D}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{E2B0E8AA-A2DA-4D30-8834-36D20A8CC477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A7D93A6-4B1F-46C6-830D-016FCF696952}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{39ED1F32-22C4-4727-87DE-A1241A62ACDB}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="241">
   <si>
     <t>Model</t>
   </si>
@@ -733,7 +733,16 @@
     <t>Targeted noxious weeds</t>
   </si>
   <si>
-    <t>Targeted knapweed</t>
+    <t>Targeted knapweed (2,4-D)</t>
+  </si>
+  <si>
+    <t>2,4-D; imazapic; glyphosate</t>
+  </si>
+  <si>
+    <t>Imazapic</t>
+  </si>
+  <si>
+    <t>Glyphosate, imazapic</t>
   </si>
 </sst>
 </file>
@@ -1874,7 +1883,7 @@
         <v>1.6916666666666667</v>
       </c>
     </row>
-    <row r="3" spans="1:44" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:44" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>43</v>
       </c>
@@ -2094,7 +2103,7 @@
         <v>0.2673611111111111</v>
       </c>
     </row>
-    <row r="5" spans="1:44" ht="216" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:44" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>43</v>
       </c>
@@ -2208,7 +2217,9 @@
       <c r="C6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>238</v>
+      </c>
       <c r="E6" s="2">
         <v>50661</v>
       </c>
@@ -2322,7 +2333,9 @@
       <c r="C7" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D7" s="3"/>
+      <c r="D7" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E7" s="2">
         <v>50730</v>
       </c>
@@ -2422,7 +2435,7 @@
         <v>3.2638888888888891E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:44" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:44" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>43</v>
       </c>
@@ -2432,7 +2445,9 @@
       <c r="C8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E8" s="2">
         <v>51025</v>
       </c>
@@ -2534,7 +2549,9 @@
       <c r="C9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E9" s="2">
         <v>54109</v>
       </c>
@@ -2760,7 +2777,9 @@
       <c r="C11" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E11" s="2">
         <v>57018</v>
       </c>
@@ -2864,7 +2883,9 @@
       <c r="C12" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>240</v>
+      </c>
       <c r="E12" s="2">
         <v>57035</v>
       </c>
@@ -3070,7 +3091,7 @@
         <v>0.79513888888888884</v>
       </c>
     </row>
-    <row r="14" spans="1:44" ht="288" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:44" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>43</v>
       </c>
@@ -3080,7 +3101,9 @@
       <c r="C14" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E14" s="2">
         <v>69625</v>
       </c>
@@ -3190,7 +3213,9 @@
       <c r="C15" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E15" s="2">
         <v>69661</v>
       </c>
@@ -3288,7 +3313,7 @@
         <v>1.0249999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:44" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:44" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>43</v>
       </c>
@@ -3504,7 +3529,7 @@
         <v>2.1041666666666665</v>
       </c>
     </row>
-    <row r="18" spans="1:44" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:44" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>43</v>
       </c>
@@ -3612,7 +3637,7 @@
         <v>1.8784722222222223</v>
       </c>
     </row>
-    <row r="19" spans="1:44" ht="388.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:44" ht="216" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>43</v>
       </c>
@@ -3724,7 +3749,7 @@
         <v>1.6048611111111111</v>
       </c>
     </row>
-    <row r="20" spans="1:44" ht="72" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:44" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>43</v>
       </c>
@@ -3734,7 +3759,9 @@
       <c r="C20" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E20" s="2">
         <v>71274</v>
       </c>
@@ -3836,7 +3863,7 @@
         <v>0.65416666666666667</v>
       </c>
     </row>
-    <row r="21" spans="1:44" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:44" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>43</v>
       </c>
@@ -3944,7 +3971,7 @@
         <v>0.71875</v>
       </c>
     </row>
-    <row r="22" spans="1:44" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:44" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
@@ -3954,7 +3981,9 @@
       <c r="C22" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="3"/>
+      <c r="D22" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E22" s="2">
         <v>71513</v>
       </c>
@@ -4162,7 +4191,7 @@
         <v>1.788888888888889</v>
       </c>
     </row>
-    <row r="24" spans="1:44" ht="244.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:44" ht="144" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>43</v>
       </c>
@@ -4272,7 +4301,7 @@
         <v>1.3868055555555556</v>
       </c>
     </row>
-    <row r="25" spans="1:44" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:44" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>43</v>
       </c>
@@ -4380,7 +4409,7 @@
         <v>2.2562500000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:44" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:44" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>43</v>
       </c>

</xml_diff>